<commit_message>
Audit full Day 13 requirements and align pilot economics, roadmap and slide
</commit_message>
<xml_diff>
--- a/Neiv_CS13.xlsx
+++ b/Neiv_CS13.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AIthucchien\track1\day13\Neiv-AI-Roadmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D07B0708-641D-40C2-B452-EB60B11B0BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{161DA9B6-810B-4077-A2B6-8A984CC8F1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5136" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -736,12 +736,6 @@
     <t>Kế toán viên công ty duyệt mọi cờ + mẫu 10% tổng việc từ phần không cờ. Chị Hạnh kiểm 1% hóa đơn thật tuần đầu, nằm trong mẫu này.</t>
   </si>
   <si>
-    <t>Giữ cổng hồ sơ: đạt quy về thực tế ≥95%, 0 lỗi nghiêm trọng, 0 tầng tụt, kappa ≥0,6 trên đủ 40 ca. Chị Hạnh/anh Tùng xác nhận. Chạy thử ≥1.000 hóa đơn, kiểm mẫu ≥200, cờ thừa ≤10% tổng việc.</t>
-  </si>
-  <si>
-    <t>Bản 2 đã phát hành: 97,3%, 0 lỗi, 0 tầng tụt, kappa 0,90. Gắn nhãn AI, quyền dữ liệu, nhật ký thay đổi, chặn MST/tiền bất nhất. Tỷ lệ duyệt 20% là giả định, tăng nếu cờ tăng.</t>
-  </si>
-  <si>
     <t>0–3 tháng, rà ngày 30. Thử ở văn phòng hiện có.</t>
   </si>
   <si>
@@ -751,9 +745,6 @@
     <t>Kế toán viên công ty duyệt mọi cờ; dự kiến 5% tổng việc gắn cờ + 5% tổng việc lấy mẫu không cờ. Hạnh xác nhận ngoại lệ.</t>
   </si>
   <si>
-    <t>Sau sửa/đổi bản: chạy lại 40 ca, giữ ≥95%, 0 lỗi nghiêm trọng, 0 tầng tụt, kappa ≥0,6. Kiểm độc lập ≥300 hóa đơn thật có đủ 4 tầng: 0 lỗi MST/tiền, đạt quy về thực tế ≥95%. Hạnh ký cổng, Tùng đối chiếu.</t>
-  </si>
-  <si>
     <t>Hoàn tất dịch vụ MST, timeout phải chặn, truy vết và quay lui. Kiểm mẫu 300 bằng nhân sự công ty; chuyên gia xử lý bất đồng. Tỷ lệ duyệt 10% chỉ dùng khi cờ ≤5%; vượt thì tăng duyệt.</t>
   </si>
   <si>
@@ -769,15 +760,9 @@
     <t>Chưa cam kết: 0 lỗi MST/tiền trên ≥1.000 hóa đơn kiểm trong ≥4 tuần; bộ 40 ca đạt ≥95%, 0 tầng tụt, kappa ≥0,6. Cờ ≤2% tổng việc. Hạnh xác nhận; lãnh đạo duyệt sau kiểm chi phí.</t>
   </si>
   <si>
-    <t>Đủ dữ liệu theo từng tầng, cảnh báo, hoàn tác và người trực. Phải có kế hoạch kinh phí kiểm mẫu bổ sung. 0/1.000 chỉ cho giới hạn gần đúng 0,3% ở 95%, không bảo đảm tuyệt đối.</t>
-  </si>
-  <si>
     <t>Khám phá tháng 6–12, giữ Mức 2 nếu thiếu bằng chứng.</t>
   </si>
   <si>
-    <t>Đọc ảnh và gắn cờ (việc 1–2); tận dụng nhập tệp gốc (3), tích hợp tra cứu MST (4) làm điều kiện an toàn.</t>
-  </si>
-  <si>
     <t>Ổn định đối chiếu MST và xử lý ngoại lệ; mở Mức 2 nếu qua cổng. Chỉ tuyển thêm văn phòng khi có người duyệt và kinh phí.</t>
   </si>
   <si>
@@ -802,9 +787,6 @@
     <t>Tháng 9: ≥100 bút toán, giảm ≥30% phút/bút toán, chấp thuận ≥90%. Mức 3 cần 0 lỗi nghiêm trọng/1.000 hóa đơn kiểm trong ≥4 tuần.</t>
   </si>
   <si>
-    <t>Mức 1: duyệt dự kiến 20%; mọi cờ + mẫu không trùng. Lùi Mức 0 khi có lỗi nghiêm trọng.</t>
-  </si>
-  <si>
     <t>Mức 2: duyệt dự kiến 10%; mọi cờ + mẫu không trùng; nếu cờ tăng thì tăng duyệt, không bỏ cờ.</t>
   </si>
   <si>
@@ -814,60 +796,21 @@
     <t>Cổng Mức 1 trang 2: bộ 40 ca ≥95%, 0 lỗi nghiêm trọng, 0 tầng tụt, kappa ≥0,6; kiểm ≥200/1.000 hóa đơn thử. Hạnh/Tùng xác nhận.</t>
   </si>
   <si>
-    <t>Cổng Mức 2 trang 2: giữ cổng 40 ca + kiểm độc lập ≥300 hóa đơn đủ 4 tầng, 0 lỗi nghiêm trọng. Quy tắc 3/n: 0/300 vẫn có giới hạn trên gần 1%, không khẳng định an toàn tuyệt đối.</t>
-  </si>
-  <si>
-    <t>Cổng Mức 3 trang 2: kiểm ≥1.000, 0 lỗi tiền/MST, đủ 4 tuần; 3/n≈0,3%. Hạch toán có bộ đề riêng và người duyệt, không dùng chung cổng đọc ảnh.</t>
-  </si>
-  <si>
-    <t>Quyền dùng dữ liệu, ẩn thông tin không cần, phân quyền/nhật ký/hoàn tác, thông báo AI. Hạnh ≤3 giờ/tuần; vòng 40 ca tốn 8,5 giờ nên chia ≥3 tuần, Tùng hỗ trợ theo lịch xác nhận. Duyệt 20% ×12.000×1,5 phút=60 giờ công ty/tháng.</t>
-  </si>
-  <si>
     <t>Xác nhận giờ Tùng, ngân sách dịch vụ MST/phần mềm và nhân sự duyệt. 10% ×12.000×1,5 phút=30 giờ/tháng, chưa kể chấm cổng độc lập. Kiểm 300 ca tối thiểu 7,5 giờ ở mức rà nhanh; ca khó cần thêm giờ.</t>
   </si>
   <si>
     <t>Xin dữ liệu hạch toán có phép, tạo nhãn/bộ đề và kinh phí kiểm ≥1.000 ca (ít nhất 25 giờ rà nhanh). Xác nhận khả năng cung cấp chuyên gia trước mọi mở rộng. Rà soát nghĩa vụ pháp lý trước phát hành.</t>
   </si>
   <si>
-    <t>Giữ số liệu đề: AI 254đ + khác 200đ +20%×1,5×50.000/60=704đ/việc; 1.760 việc, 3,97 triệu/khách/tháng: biên 68,79%. Mức 0:1.704đ, biên 24,46%. Doanh thu tập trung; kịch bản xấu hết tiền tháng 7. Phí mua chưa báo giá.</t>
-  </si>
-  <si>
-    <t>Mức 2:579đ/việc, biên 74,33% với 3,97 triệu và 1.760 việc. Nếu doanh thu còn 3,71 triệu, biên ≈72,53%. Cần kiểm phí mua và lượng việc thực tế; 12.000 việc/văn phòng thử không được thay cho 1.760 việc/khách giả định.</t>
-  </si>
-  <si>
     <t>Mức 3:516,5đ/việc, biên 77,10% theo đề, chưa gồm chi phí mua phát sinh vượt 200đ. Trước tháng 7 phải có hợp đồng/nguồn tiền hoặc giảm phạm vi vì kịch bản hết tiền tháng 7. Không suy lợi nhuận từ mẫu nhỏ.</t>
   </si>
   <si>
-    <t>NẾU phát hiện ≥1 lỗi MST/tiền lúc nào THÌ dừng tự nhập và lùi Mức 0. NẾU ngày 30 cờ thừa &gt;10%/1.000 ca hoặc thời gian giảm &lt;50%/100 ảnh THÌ sửa, giữ quy mô. NẾU ARPA &lt;3,71 triệu trong 2 tháng liên tiếp trên ≥10 văn phòng THÌ dừng mở rộng; chưa đủ 10 thì chưa kết luận.</t>
-  </si>
-  <si>
-    <t>NẾU ngày 90 không đủ 300 ca kiểm hoặc có ≥1 lỗi MST/tiền THÌ giữ/lùi mức và sửa. NẾU doanh thu &lt;3,71 triệu/văn phòng trong 2 tháng, trên ≥10 văn phòng THÌ dừng mở rộng. Kiểm hàng tháng, thiếu mẫu thì giữ thử nghiệm.</t>
-  </si>
-  <si>
-    <t>NẾU tháng 6 chưa có dữ liệu/bộ đề hạch toán THÌ tiếp tục Chờ và xem lại tháng 9. NẾU tháng 9 gợi ý chấp thuận &lt;90%/100 bút toán THÌ dừng nhánh. NẾU thiếu kinh phí trước tháng 7 THÌ dừng tuyển mới, xử lý nghĩa vụ hiện có.</t>
-  </si>
-  <si>
-    <t>Ngày 30: phút/100 ảnh và 100 tệp so với thủ công, cờ thừa/1.000, mẫu ≥200, lỗi MST/tiền; chi phí duyệt thực.</t>
-  </si>
-  <si>
-    <t>Đi tiếp Mức 1 nếu đạt mục tiêu; sửa khi giảm giờ &lt;50% hoặc cờ thừa &gt;10%; ≥1 lỗi nghiêm trọng thì dừng tự nhập ngay. Chưa đủ mẫu thì giữ thử nghiệm.</t>
-  </si>
-  <si>
     <t>Hạnh xác nhận chất lượng, Tùng đối chiếu; lãnh đạo sản phẩm quyết phạm vi.</t>
   </si>
   <si>
-    <t>Ngày 60: bộ 40 ca hồi quy, 300 hóa đơn kiểm tích lũy, tỷ lệ duyệt, chi phí mua; ARPA 2 tháng nếu đã có ≥10 văn phòng.</t>
-  </si>
-  <si>
-    <t>Sửa/giữ mức nếu thiếu mẫu hoặc không đạt cổng. Dừng mở rộng nếu ARPA &lt;3,71 triệu trong 2 tháng và ≥10 văn phòng; chưa đủ 10 thì không coi là đạt.</t>
-  </si>
-  <si>
     <t>Hạnh ký cổng, kỹ sư xác nhận chặn/hoàn tác; lãnh đạo sản phẩm và tài chính quyết.</t>
   </si>
   <si>
-    <t>Ngày 90: đủ cổng Mức 2, 0 lỗi/300 hóa đơn kiểm, biên thực ≥60%, doanh thu và số văn phòng; khả năng tiền trước tháng 7.</t>
-  </si>
-  <si>
     <t>Đi tiếp Mức 2 khi đủ mọi cổng. Thiếu bằng chứng: giữ Mức 1; sai tiền/MST: dừng tự nhập. Đổi hướng sang tích hợp nếu phí mua làm biên &lt;60% và không giảm được an toàn.</t>
   </si>
   <si>
@@ -877,9 +820,6 @@
     <t>So bản mới trên toàn bộ 40 ca, kiểm đủ 4 tầng, ≥95%, 0 lỗi, 0 tầng tụt; tính lại chi phí gọi và duyệt, thời gian đáp ứng.</t>
   </si>
   <si>
-    <t>Chỉ đổi mô hình sau cổng và kế hoạch quay lui. Giá rẻ không đủ lý do tự tăng mức. Nếu kém chất lượng thì giữ bản đã qua cổng.</t>
-  </si>
-  <si>
     <t>Kỹ sư chạy kiểm, Hạnh/Tùng chấm; lãnh đạo sản phẩm duyệt đổi.</t>
   </si>
   <si>
@@ -901,19 +841,79 @@
     <t>Người phụ trách pháp lý/dữ liệu được chỉ định và lãnh đạo sản phẩm.</t>
   </si>
   <si>
-    <t>Đề xuất triển khai SổSạch ở Mức 1, duyệt 20% hóa đơn, mục tiêu giảm 50% giờ nhập ảnh. Chỉ lên Mức 2 khi qua cổng chất lượng, rà soát quyết định ngày 90.</t>
-  </si>
-  <si>
-    <t>0–3 tháng: đọc ảnh và gắn cờ. 3–6 tháng: đối chiếu mã số thuế, tích hợp dịch vụ sẵn có. 6–12 tháng: mở rộng có điều kiện, khám phá hạch toán khi đủ dữ liệu.</t>
-  </si>
-  <si>
-    <t>Cần bộ đề 40 hóa đơn, quyền dùng dữ liệu và kết nối phần mềm. Chị Hạnh tối đa 3 giờ/tuần, anh Tùng hỗ trợ chấm. Công ty bố trí 60 giờ duyệt/tháng cho 12.000 hóa đơn. Mức 1: 704 đồng/việc, biên gộp 68,79% theo giả định đề.</t>
-  </si>
-  <si>
-    <t>Sai mã số thuế hoặc tiền: ngừng tự nhập ngay. Duyệt mọi cờ và lấy mẫu. Nếu doanh thu dưới 3,71 triệu/văn phòng trong 2 tháng, với ít nhất 10 văn phòng, dừng mở rộng. Chưa đủ mẫu thì giữ thử nghiệm, lưu ý kịch bản hết tiền tháng 7.</t>
-  </si>
-  <si>
-    <t>Ngày 30/60/90 từ lúc bắt đầu: xem lỗi, cờ thừa, giờ nhập và chi phí. Mức 2 cần 0 lỗi nghiêm trọng/300 hóa đơn kiểm tra, đạt từ 95%, không tầng tụt. Mô hình, giá hoặc quy định đổi: rà soát ngay. Các ngưỡng mới là đề xuất cần kiểm chứng.</t>
+    <t>Giữ cổng hồ sơ: đạt quy về thực tế ≥95%, 0 lỗi nghiêm trọng, 0 tầng tụt, kappa ≥0,6 trên 40 ca; Hạnh/Tùng xác nhận. Thử ≤1.000 hóa đơn, kiểm ≥200 gồm mọi cờ + mẫu không cờ. Cờ thừa ≤10% tổng việc. Chỉ tự nhập sau đối chiếu MST/tiền; hết ngân sách chưa qua cổng thì giữ Mức 0.</t>
+  </si>
+  <si>
+    <t>Bản 2 đã phát hành: 97,3%, 0 lỗi, 0 tầng tụt, kappa 0,90. Tích hợp tra cứu MST trước tự nhập; lỗi tra cứu thì chặn. Cần quyền dữ liệu, thông báo AI, phân quyền, nhật ký và hoàn tác. Duyệt 20% là giả định, tăng khi cờ tăng. Thử 1.000 ca: 5 giờ duyệt, 704.000đ chi phí biến đổi dự kiến; duyệt riêng phí phát sinh.</t>
+  </si>
+  <si>
+    <t>Sau sửa/đổi bản: chạy lại 40 ca, giữ ≥95%, 0 lỗi nghiêm trọng, 0 tầng tụt, kappa ≥0,6. Kiểm độc lập ≥300 hóa đơn thật: 0 lỗi MST/tiền, đạt quy về thực tế ≥95%. Có mẫu ngẫu nhiên đại diện, tăng mẫu các tầng hiếm và báo riêng. Hạnh ký cổng, Tùng đối chiếu.</t>
+  </si>
+  <si>
+    <t>Đủ dữ liệu theo tầng, cảnh báo, hoàn tác, người trực và kinh phí kiểm mẫu bổ sung. Quy tắc 3/n chỉ là gần đúng với mẫu ngẫu nhiên độc lập, không áp thẳng cho bộ đề chọn ca có chủ đích; 0 lỗi không bảo đảm an toàn tuyệt đối. Thiếu bằng chứng thì giữ Mức 2.</t>
+  </si>
+  <si>
+    <t>Ngày 30: hoàn tất đọc ảnh và gắn cờ (1–2), tận dụng bộ nhập tệp gốc (3), tích hợp MST (4) trước tự nhập. Thử tối đa 1.000 hóa đơn tại văn phòng hiện có; ngày 90 quyết định bước tiếp sau cổng.</t>
+  </si>
+  <si>
+    <t>Mức 0 khi chưa tích hợp đối chiếu MST/tiền hoặc chưa duyệt ngân sách. Mức 1 dự kiến duyệt 20%, mọi cờ + mẫu không trùng. Lùi Mức 0 khi có lỗi nghiêm trọng. Ngày 90 chỉ xét Mức 2 nếu đủ 300 ca kiểm độc lập.</t>
+  </si>
+  <si>
+    <t>Cổng Mức 2: giữ cổng 40 ca và kiểm độc lập ≥300 hóa đơn thật, 0 lỗi nghiêm trọng. Lấy mẫu ngẫu nhiên đại diện, bổ sung ca tầng hiếm. Quy tắc 3/n≈1% chỉ gần đúng cho phần mẫu ngẫu nhiên độc lập; bộ đề chủ đích không chứng minh tỷ lệ lỗi thật. Hạnh xác nhận.</t>
+  </si>
+  <si>
+    <t>Cổng Mức 3: ≥1.000 ca kiểm, 0 lỗi tiền/MST trong ≥4 tuần và không tầng tụt. 3/n≈0,3% chỉ áp gần đúng với mẫu ngẫu nhiên độc lập. Ghi kết quả từng tầng, bổ sung ca hiếm. Hạch toán cần bộ đề riêng và người duyệt.</t>
+  </si>
+  <si>
+    <t>Quyền dữ liệu, phân quyền/nhật ký/hoàn tác và thông báo AI. Hạnh ≤3 giờ/tuần, Tùng hỗ trợ theo lịch cần xác nhận. Vòng 40 ca 8,5 giờ: xếp ≥3 tuần, dành giờ cho kiểm 1% tuần đầu. Thử 1.000 ca cần 5 giờ duyệt công ty; toàn bộ 12.000 ca cần 60 giờ/tháng và gói giá/ngân sách riêng.</t>
+  </si>
+  <si>
+    <t>Theo bình quân đề: 704đ/việc ở Mức 1, 1.760 việc và doanh thu 3,97 triệu: biên 68,79%. Thử 1.000 ca: chi phí biến đổi dự kiến 704.000đ; phí phát sinh duyệt riêng. 12.000 ca tốn 8,448 triệu/tháng, không áp biên 68,79% cho mức này. Doanh thu tập trung; kịch bản xấu hết tiền tháng 7.</t>
+  </si>
+  <si>
+    <t>Mức 2:579đ/việc, biên 74,33% với 3,97 triệu và 1.760 việc; tại doanh thu 3,71 triệu biên ≈72,53%. Nếu xử lý 12.000 ca, chi phí 6,948 triệu/tháng, cần giá ≥17,37 triệu để biên 60% trước phí phát sinh. Phải duyệt gói giá/hạn mức và ngân sách trước mở quy mô.</t>
+  </si>
+  <si>
+    <t>NẾU có ≥1 lỗi MST/tiền bất kỳ lúc nào THÌ dừng tự nhập, lùi Mức 0. NẾU ngày 30 cờ thừa &gt;10%/1.000 ca hoặc giảm giờ &lt;50%/100 ảnh THÌ sửa, giữ quy mô. Thử đủ 1.000 ca mà chưa qua cổng: không tăng phạm vi. Rà hàng tháng: ARPA &lt;3,71 triệu trong 2 tháng liên tiếp trên ≥10 văn phòng thì dừng mở rộng; thiếu mẫu thì chưa kết luận.</t>
+  </si>
+  <si>
+    <t>NẾU ngày 90 chưa đủ 300 ca kiểm hoặc có ≥1 lỗi MST/tiền THÌ giữ/lùi mức và sửa. Rà mỗi tháng: doanh thu &lt;3,71 triệu/văn phòng trong 2 tháng liên tiếp trên ≥10 văn phòng thì dừng mở rộng; thiếu mẫu thì giữ thử nghiệm. Chưa chốt giá/hạn mức hoặc kinh phí thì không xử lý toàn bộ 12.000 ca.</t>
+  </si>
+  <si>
+    <t>NẾU tháng 6 thiếu dữ liệu/bộ đề hạch toán THÌ tiếp tục Chờ, xem lại tháng 9. NẾU tháng 9 chấp thuận &lt;90%/100 bút toán THÌ dừng nhánh. NẾU trước tháng 7 thiếu kinh phí THÌ dừng tuyển mới. Tiếp tục rà hàng tháng: ARPA &lt;3,71 triệu trong 2 tháng liên tiếp trên ≥10 văn phòng thì dừng mở rộng.</t>
+  </si>
+  <si>
+    <t>Ngày 30: tổng phút/100 ảnh và 100 tệp so với thủ công, cờ thừa/1.000, mẫu ≥200, lỗi MST/tiền và chi phí thực. Cờ thừa = số ca gắn cờ được kế toán xác nhận không cần can thiệp / tổng ca xử lý. Rà ngân sách 704.000đ cho 1.000 ca, tách phí phát sinh.</t>
+  </si>
+  <si>
+    <t>Đi tiếp Mức 1 nếu đạt mục tiêu và đủ ngân sách; giảm giờ &lt;50% hoặc cờ thừa &gt;10% thì sửa, giữ phạm vi. ≥1 lỗi nghiêm trọng thì dừng tự nhập ngay. Đủ 1.000 ca chưa qua cổng hoặc chưa có giá/hạn mức thì không mở rộng.</t>
+  </si>
+  <si>
+    <t>Ngày 90: cổng Mức 2, 0 lỗi/300 hóa đơn kiểm, biên thực ≥60%, doanh thu và số văn phòng. Kiểm khả năng tiền trước tháng 7. Chỉ xử lý 12.000 ca khi có gói giá/hạn mức hoặc kinh phí thử riêng được duyệt.</t>
+  </si>
+  <si>
+    <t>Chỉ đổi sau cổng, so chi phí và có phương án quay lui. Xem lại rủi ro bị nuốt, chấm lại việc bị ảnh hưởng, ghi lý do đổi thứ tự. Báo người dùng khi hành vi đổi và theo dõi khiếu nại 2 tuần. Giá rẻ không đủ lý do tăng mức.</t>
+  </si>
+  <si>
+    <t>Đề xuất thử nghiệm SổSạch cho văn phòng kế toán ở Mức 1 trên 1.000 hóa đơn, duyệt 20%, mục tiêu giảm 50% giờ nhập ảnh và quyết định lên Mức 2 vào ngày 90 nếu qua cổng chất lượng.</t>
+  </si>
+  <si>
+    <t>0–3 tháng: đọc ảnh, gắn cờ và đối chiếu mã số thuế. 3–6 tháng: giảm tỷ lệ duyệt sau cổng Mức 2. 6–12 tháng: mở rộng có điều kiện, khám phá hạch toán khi đủ dữ liệu.</t>
+  </si>
+  <si>
+    <t>Cần bộ đề 40 hóa đơn, quyền dữ liệu và kết nối phần mềm. Hạnh tối đa 3 giờ/tuần, Tùng hỗ trợ chấm. Công ty cần 5 giờ duyệt/1.000 hóa đơn, chi phí dự kiến 704.000 đồng. Biên 68,79% chỉ theo bình quân đề. Phí tích hợp cần duyệt riêng.</t>
+  </si>
+  <si>
+    <t>Rủi ro lớn nhất: 65% doanh thu từ 30% văn phòng. Theo dõi từ thử nghiệm, dừng mở rộng nếu doanh thu dưới 3,71 triệu/văn phòng trong 2 tháng liên tiếp trên ít nhất 10 văn phòng. Chưa đủ mẫu thì giữ thử nghiệm. Kịch bản xấu hết tiền tháng 7.</t>
+  </si>
+  <si>
+    <t>Ngày 30/60/90 và khi mô hình, giá hoặc quy định đổi: rà soát. Mức 2 cần đạt từ 95%, không tầng tụt, 0 lỗi nghiêm trọng/300 hóa đơn kiểm. Có 1 lỗi mã số thuế/tiền: ngừng tự nhập ngay. Ngưỡng mới cần kiểm chứng.</t>
+  </si>
+  <si>
+    <t>Ngày 60: bộ 40 ca hồi quy, 300 hóa đơn kiểm tích lũy, tỷ lệ duyệt và chi phí mua. Đo ARPA từng tháng, xét 2 tháng liên tiếp nếu đã có ≥10 văn phòng. Thiếu mẫu, giờ chấm hoặc kinh phí kiểm độc lập thì giữ quy mô thử.</t>
+  </si>
+  <si>
+    <t>Sửa/giữ mức khi thiếu mẫu hoặc không đạt cổng. Dừng mở rộng nếu ARPA &lt;3,71 triệu/văn phòng trong 2 tháng liên tiếp trên ≥10 văn phòng; chưa đủ 10 thì chưa kết luận. Không tăng quyền tự động chỉ vì tới ngày 60.</t>
   </si>
 </sst>
 </file>
@@ -2281,7 +2281,7 @@
         <v>Dưới ngưỡng</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="72" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A6" s="10">
         <v>1</v>
       </c>
@@ -2295,13 +2295,13 @@
         <v>230</v>
       </c>
       <c r="E6" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="G6" s="7" t="s">
         <v>231</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>233</v>
       </c>
       <c r="H6" s="14">
         <v>0.2</v>
@@ -2326,7 +2326,7 @@
         <v>Có</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="72" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="10">
         <v>2</v>
       </c>
@@ -2334,19 +2334,19 @@
         <v>74</v>
       </c>
       <c r="C7" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>235</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>238</v>
       </c>
       <c r="H7" s="14">
         <v>0.1</v>
@@ -2371,7 +2371,7 @@
         <v>Có</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="72" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A8" s="10">
         <v>3</v>
       </c>
@@ -2379,19 +2379,19 @@
         <v>75</v>
       </c>
       <c r="C8" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>237</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="G8" s="7" t="s">
         <v>239</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>242</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>243</v>
       </c>
       <c r="H8" s="14">
         <v>0.05</v>
@@ -2577,18 +2577,18 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
         <v>104</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>244</v>
+        <v>270</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -2596,13 +2596,13 @@
         <v>105</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -2610,83 +2610,83 @@
         <v>44</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>107</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A10" s="23" t="s">
         <v>108</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="72" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>262</v>
+        <v>275</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>263</v>
+        <v>276</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A12" s="23" t="s">
         <v>110</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
     </row>
   </sheetData>
@@ -2729,60 +2729,60 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>117</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>118</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>119</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>120</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>277</v>
+        <v>258</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -2790,13 +2790,13 @@
         <v>121</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>282</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="57.6" x14ac:dyDescent="0.3">
@@ -2804,13 +2804,13 @@
         <v>122</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>283</v>
+        <v>263</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>284</v>
+        <v>264</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>285</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -2858,11 +2858,11 @@
         <v>128</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C4" s="25">
         <f>IF(TRIM(B4)="",0,LEN(TRIM(B4))-LEN(SUBSTITUTE(TRIM(B4)," ",""))+1)</f>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="D4" s="17" t="str">
         <f>IF(C4=0,"Trống",IF(C4&gt;60,"Quá 60 chữ","Đạt"))</f>
@@ -2874,11 +2874,11 @@
         <v>129</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C5" s="25">
         <f>IF(TRIM(B5)="",0,LEN(TRIM(B5))-LEN(SUBSTITUTE(TRIM(B5)," ",""))+1)</f>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D5" s="17" t="str">
         <f>IF(C5=0,"Trống",IF(C5&gt;60,"Quá 60 chữ","Đạt"))</f>
@@ -2890,11 +2890,11 @@
         <v>130</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C6" s="25">
         <f>IF(TRIM(B6)="",0,LEN(TRIM(B6))-LEN(SUBSTITUTE(TRIM(B6)," ",""))+1)</f>
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D6" s="17" t="str">
         <f>IF(C6=0,"Trống",IF(C6&gt;60,"Quá 60 chữ","Đạt"))</f>
@@ -2906,11 +2906,11 @@
         <v>131</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C7" s="25">
         <f>IF(TRIM(B7)="",0,LEN(TRIM(B7))-LEN(SUBSTITUTE(TRIM(B7)," ",""))+1)</f>
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="17" t="str">
         <f>IF(C7=0,"Trống",IF(C7&gt;60,"Quá 60 chữ","Đạt"))</f>
@@ -2922,11 +2922,11 @@
         <v>132</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C8" s="25">
         <f>IF(TRIM(B8)="",0,LEN(TRIM(B8))-LEN(SUBSTITUTE(TRIM(B8)," ",""))+1)</f>
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D8" s="17" t="str">
         <f>IF(C8=0,"Trống",IF(C8&gt;60,"Quá 60 chữ","Đạt"))</f>

</xml_diff>